<commit_message>
Ship Nuxt demo, xlsx preview layout with cell colors, and env limits.
Replace Vite examples with Nuxt; move Excel table rendering into @contract-kit/xlsx (mountXlsxPreview + getPreview styles); document browser/Node constraints and refresh Pages landing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/templates/采购合同.xlsx
+++ b/examples/templates/采购合同.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>采购合同</t>
   </si>
@@ -79,6 +79,12 @@
     <t>{{payMethod:select}}</t>
   </si>
   <si>
+    <t>交货区域</t>
+  </si>
+  <si>
+    <t>{{deliveryRegions:multiselect}}</t>
+  </si>
+  <si>
     <t>付款期限</t>
   </si>
   <si>
@@ -121,13 +127,19 @@
     <t>{{filledAt:display}}</t>
   </si>
   <si>
+    <t>附件图片</t>
+  </si>
+  <si>
+    <t>{{stamp:image}}</t>
+  </si>
+  <si>
     <t>序号</t>
   </si>
   <si>
     <t>货物名称</t>
   </si>
   <si>
-    <t>规格型号</t>
+    <t>类别</t>
   </si>
   <si>
     <t>数量</t>
@@ -142,7 +154,7 @@
     <t>{{items.name}}</t>
   </si>
   <si>
-    <t>{{items.spec}}</t>
+    <t>{{items.category:select}}</t>
   </si>
   <si>
     <t>{{items.qty:number}}</t>
@@ -593,7 +605,7 @@
   <sheetPr>
     <tabColor rgb="FF1B3A5C"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="18" customWidth="1"/>
@@ -786,42 +798,62 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B21" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="B22" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="B24" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="E24" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E23" s="7" t="s">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>45</v>
       </c>
+      <c r="B25" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B4:D4"/>
@@ -841,6 +873,8 @@
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B22:D22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Let definition own field type and export format, not the Word marker.
Documents only keep {{name}} anchors; outputFormat formats dates, numbers, and option labels on export while data stays canonical.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/templates/采购合同.xlsx
+++ b/examples/templates/采购合同.xlsx
@@ -70,19 +70,19 @@
     <t>合同金额（元）</t>
   </si>
   <si>
-    <t>{{amount:number}}</t>
+    <t>{{amount}}</t>
   </si>
   <si>
     <t>付款方式</t>
   </si>
   <si>
-    <t>{{payMethod:select}}</t>
+    <t>{{payMethod}}</t>
   </si>
   <si>
     <t>交货区域</t>
   </si>
   <si>
-    <t>{{deliveryRegions:multiselect}}</t>
+    <t>{{deliveryRegions}}</t>
   </si>
   <si>
     <t>付款期限</t>
@@ -94,7 +94,7 @@
     <t>交货日期</t>
   </si>
   <si>
-    <t>{{deliveryDate:date}}</t>
+    <t>{{deliveryDate}}</t>
   </si>
   <si>
     <t>交货地点</t>
@@ -112,25 +112,25 @@
     <t>签订日期</t>
   </si>
   <si>
-    <t>{{signDate:date}}</t>
+    <t>{{signDate}}</t>
   </si>
   <si>
     <t>备注说明</t>
   </si>
   <si>
-    <t>{{note:textarea}}</t>
+    <t>{{note}}</t>
   </si>
   <si>
     <t>填写日</t>
   </si>
   <si>
-    <t>{{filledAt:display}}</t>
+    <t>{{filledAt}}</t>
   </si>
   <si>
     <t>附件图片</t>
   </si>
   <si>
-    <t>{{stamp:image}}</t>
+    <t>{{stamp}}</t>
   </si>
   <si>
     <t>序号</t>
@@ -154,13 +154,13 @@
     <t>{{items.name}}</t>
   </si>
   <si>
-    <t>{{items.category:select}}</t>
-  </si>
-  <si>
-    <t>{{items.qty:number}}</t>
-  </si>
-  <si>
-    <t>{{items.unitPrice:number}}</t>
+    <t>{{items.category}}</t>
+  </si>
+  <si>
+    <t>{{items.qty}}</t>
+  </si>
+  <si>
+    <t>{{items.unitPrice}}</t>
   </si>
 </sst>
 </file>

</xml_diff>